<commit_message>
running all again with GMM and imroved kmean
</commit_message>
<xml_diff>
--- a/excercise2/clusters/cluster_evaluation_results.xlsx
+++ b/excercise2/clusters/cluster_evaluation_results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>method</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>hdbscan</t>
+  </si>
+  <si>
+    <t>gmm</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -616,6 +619,53 @@
         <v>360</v>
       </c>
     </row>
+    <row r="5" spans="1:15">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5">
+        <v>689</v>
+      </c>
+      <c r="C5">
+        <v>689</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>329</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>360</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>